<commit_message>
fix: backslash path fixes in WellsTest, CWDS xlsx and DistributionProfile
</commit_message>
<xml_diff>
--- a/input/Studies/MEET2/CycledWellDumpingSeparator.xlsx
+++ b/input/Studies/MEET2/CycledWellDumpingSeparator.xlsx
@@ -1124,7 +1124,7 @@
       </c>
       <c r="O2" s="12" t="inlineStr">
         <is>
-          <t>Production\FlashFractions\FlashFractionsTest.csv</t>
+          <t>Production/FlashFractions/FlashFractionsTest.csv</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="O3" s="12" t="inlineStr">
         <is>
-          <t>Production\FlashFractions\FlashFractionsTest.csv</t>
+          <t>Production/FlashFractions/FlashFractionsTest.csv</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -1428,6 +1428,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
         <is>
@@ -1576,6 +1577,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>

</xml_diff>